<commit_message>
refresh-countries: also rebuild PTCC template country dropdown (col J)
</commit_message>
<xml_diff>
--- a/public/files/Participant-Bulk-Import-Excel-Format-v2.xlsx
+++ b/public/files/Participant-Bulk-Import-Excel-Format-v2.xlsx
@@ -16,7 +16,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" uniqueCount="800">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" uniqueCount="803">
   <si>
     <t>S.No.</t>
   </si>
@@ -1264,6 +1264,15 @@
   </si>
   <si>
     <t>KOR</t>
+  </si>
+  <si>
+    <t>Kosovo</t>
+  </si>
+  <si>
+    <t>XK</t>
+  </si>
+  <si>
+    <t>XKX</t>
   </si>
   <si>
     <t>Kuwait</t>
@@ -3110,7 +3119,7 @@
   </sheetData>
   <dataValidations count="1">
     <dataValidation type="list" operator="between" allowBlank="1" showDropDown="0" showInputMessage="1" showErrorMessage="1" sqref="M2:M1000">
-      <formula1>'Country List'!$B$2:$B$250</formula1>
+      <formula1>'Country List'!$B$2:$B$251</formula1>
     </dataValidation>
   </dataValidations>
   <printOptions gridLines="false" gridLinesSet="true"/>
@@ -3124,7 +3133,7 @@
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
   </sheetPr>
-  <dimension ref="A1:E250"/>
+  <dimension ref="A1:E251"/>
   <sheetFormatPr defaultRowHeight="14.4" defaultColWidth="10.5" outlineLevelRow="0" outlineLevelCol="0"/>
   <sheetData>
     <row r="1" spans="1:5">
@@ -5186,7 +5195,7 @@
     </row>
     <row r="122" spans="1:5">
       <c r="A122">
-        <v>120</v>
+        <v>250</v>
       </c>
       <c r="B122" t="s">
         <v>414</v>
@@ -5198,12 +5207,12 @@
         <v>416</v>
       </c>
       <c r="E122">
-        <v>414</v>
+        <v>412</v>
       </c>
     </row>
     <row r="123" spans="1:5">
       <c r="A123">
-        <v>121</v>
+        <v>120</v>
       </c>
       <c r="B123" t="s">
         <v>417</v>
@@ -5215,12 +5224,12 @@
         <v>419</v>
       </c>
       <c r="E123">
-        <v>417</v>
+        <v>414</v>
       </c>
     </row>
     <row r="124" spans="1:5">
       <c r="A124">
-        <v>122</v>
+        <v>121</v>
       </c>
       <c r="B124" t="s">
         <v>420</v>
@@ -5232,12 +5241,12 @@
         <v>422</v>
       </c>
       <c r="E124">
-        <v>418</v>
+        <v>417</v>
       </c>
     </row>
     <row r="125" spans="1:5">
       <c r="A125">
-        <v>123</v>
+        <v>122</v>
       </c>
       <c r="B125" t="s">
         <v>423</v>
@@ -5249,12 +5258,12 @@
         <v>425</v>
       </c>
       <c r="E125">
-        <v>428</v>
+        <v>418</v>
       </c>
     </row>
     <row r="126" spans="1:5">
       <c r="A126">
-        <v>124</v>
+        <v>123</v>
       </c>
       <c r="B126" t="s">
         <v>426</v>
@@ -5266,12 +5275,12 @@
         <v>428</v>
       </c>
       <c r="E126">
-        <v>422</v>
+        <v>428</v>
       </c>
     </row>
     <row r="127" spans="1:5">
       <c r="A127">
-        <v>125</v>
+        <v>124</v>
       </c>
       <c r="B127" t="s">
         <v>429</v>
@@ -5283,12 +5292,12 @@
         <v>431</v>
       </c>
       <c r="E127">
-        <v>426</v>
+        <v>422</v>
       </c>
     </row>
     <row r="128" spans="1:5">
       <c r="A128">
-        <v>126</v>
+        <v>125</v>
       </c>
       <c r="B128" t="s">
         <v>432</v>
@@ -5300,12 +5309,12 @@
         <v>434</v>
       </c>
       <c r="E128">
-        <v>430</v>
+        <v>426</v>
       </c>
     </row>
     <row r="129" spans="1:5">
       <c r="A129">
-        <v>127</v>
+        <v>126</v>
       </c>
       <c r="B129" t="s">
         <v>435</v>
@@ -5317,12 +5326,12 @@
         <v>437</v>
       </c>
       <c r="E129">
-        <v>434</v>
+        <v>430</v>
       </c>
     </row>
     <row r="130" spans="1:5">
       <c r="A130">
-        <v>128</v>
+        <v>127</v>
       </c>
       <c r="B130" t="s">
         <v>438</v>
@@ -5334,12 +5343,12 @@
         <v>440</v>
       </c>
       <c r="E130">
-        <v>438</v>
+        <v>434</v>
       </c>
     </row>
     <row r="131" spans="1:5">
       <c r="A131">
-        <v>129</v>
+        <v>128</v>
       </c>
       <c r="B131" t="s">
         <v>441</v>
@@ -5351,12 +5360,12 @@
         <v>443</v>
       </c>
       <c r="E131">
-        <v>440</v>
+        <v>438</v>
       </c>
     </row>
     <row r="132" spans="1:5">
       <c r="A132">
-        <v>130</v>
+        <v>129</v>
       </c>
       <c r="B132" t="s">
         <v>444</v>
@@ -5368,12 +5377,12 @@
         <v>446</v>
       </c>
       <c r="E132">
-        <v>442</v>
+        <v>440</v>
       </c>
     </row>
     <row r="133" spans="1:5">
       <c r="A133">
-        <v>131</v>
+        <v>130</v>
       </c>
       <c r="B133" t="s">
         <v>447</v>
@@ -5385,12 +5394,12 @@
         <v>449</v>
       </c>
       <c r="E133">
-        <v>446</v>
+        <v>442</v>
       </c>
     </row>
     <row r="134" spans="1:5">
       <c r="A134">
-        <v>133</v>
+        <v>131</v>
       </c>
       <c r="B134" t="s">
         <v>450</v>
@@ -5402,12 +5411,12 @@
         <v>452</v>
       </c>
       <c r="E134">
-        <v>450</v>
+        <v>446</v>
       </c>
     </row>
     <row r="135" spans="1:5">
       <c r="A135">
-        <v>134</v>
+        <v>133</v>
       </c>
       <c r="B135" t="s">
         <v>453</v>
@@ -5419,12 +5428,12 @@
         <v>455</v>
       </c>
       <c r="E135">
-        <v>454</v>
+        <v>450</v>
       </c>
     </row>
     <row r="136" spans="1:5">
       <c r="A136">
-        <v>135</v>
+        <v>134</v>
       </c>
       <c r="B136" t="s">
         <v>456</v>
@@ -5436,12 +5445,12 @@
         <v>458</v>
       </c>
       <c r="E136">
-        <v>458</v>
+        <v>454</v>
       </c>
     </row>
     <row r="137" spans="1:5">
       <c r="A137">
-        <v>136</v>
+        <v>135</v>
       </c>
       <c r="B137" t="s">
         <v>459</v>
@@ -5453,12 +5462,12 @@
         <v>461</v>
       </c>
       <c r="E137">
-        <v>462</v>
+        <v>458</v>
       </c>
     </row>
     <row r="138" spans="1:5">
       <c r="A138">
-        <v>137</v>
+        <v>136</v>
       </c>
       <c r="B138" t="s">
         <v>462</v>
@@ -5470,12 +5479,12 @@
         <v>464</v>
       </c>
       <c r="E138">
-        <v>466</v>
+        <v>462</v>
       </c>
     </row>
     <row r="139" spans="1:5">
       <c r="A139">
-        <v>138</v>
+        <v>137</v>
       </c>
       <c r="B139" t="s">
         <v>465</v>
@@ -5487,12 +5496,12 @@
         <v>467</v>
       </c>
       <c r="E139">
-        <v>470</v>
+        <v>466</v>
       </c>
     </row>
     <row r="140" spans="1:5">
       <c r="A140">
-        <v>139</v>
+        <v>138</v>
       </c>
       <c r="B140" t="s">
         <v>468</v>
@@ -5504,12 +5513,12 @@
         <v>470</v>
       </c>
       <c r="E140">
-        <v>584</v>
+        <v>470</v>
       </c>
     </row>
     <row r="141" spans="1:5">
       <c r="A141">
-        <v>140</v>
+        <v>139</v>
       </c>
       <c r="B141" t="s">
         <v>471</v>
@@ -5521,12 +5530,12 @@
         <v>473</v>
       </c>
       <c r="E141">
-        <v>474</v>
+        <v>584</v>
       </c>
     </row>
     <row r="142" spans="1:5">
       <c r="A142">
-        <v>141</v>
+        <v>140</v>
       </c>
       <c r="B142" t="s">
         <v>474</v>
@@ -5538,12 +5547,12 @@
         <v>476</v>
       </c>
       <c r="E142">
-        <v>478</v>
+        <v>474</v>
       </c>
     </row>
     <row r="143" spans="1:5">
       <c r="A143">
-        <v>142</v>
+        <v>141</v>
       </c>
       <c r="B143" t="s">
         <v>477</v>
@@ -5555,12 +5564,12 @@
         <v>479</v>
       </c>
       <c r="E143">
-        <v>480</v>
+        <v>478</v>
       </c>
     </row>
     <row r="144" spans="1:5">
       <c r="A144">
-        <v>143</v>
+        <v>142</v>
       </c>
       <c r="B144" t="s">
         <v>480</v>
@@ -5572,12 +5581,12 @@
         <v>482</v>
       </c>
       <c r="E144">
-        <v>175</v>
+        <v>480</v>
       </c>
     </row>
     <row r="145" spans="1:5">
       <c r="A145">
-        <v>144</v>
+        <v>143</v>
       </c>
       <c r="B145" t="s">
         <v>483</v>
@@ -5589,12 +5598,12 @@
         <v>485</v>
       </c>
       <c r="E145">
-        <v>484</v>
+        <v>175</v>
       </c>
     </row>
     <row r="146" spans="1:5">
       <c r="A146">
-        <v>145</v>
+        <v>144</v>
       </c>
       <c r="B146" t="s">
         <v>486</v>
@@ -5606,12 +5615,12 @@
         <v>488</v>
       </c>
       <c r="E146">
-        <v>583</v>
+        <v>484</v>
       </c>
     </row>
     <row r="147" spans="1:5">
       <c r="A147">
-        <v>146</v>
+        <v>145</v>
       </c>
       <c r="B147" t="s">
         <v>489</v>
@@ -5623,12 +5632,12 @@
         <v>491</v>
       </c>
       <c r="E147">
-        <v>498</v>
+        <v>583</v>
       </c>
     </row>
     <row r="148" spans="1:5">
       <c r="A148">
-        <v>147</v>
+        <v>146</v>
       </c>
       <c r="B148" t="s">
         <v>492</v>
@@ -5640,12 +5649,12 @@
         <v>494</v>
       </c>
       <c r="E148">
-        <v>492</v>
+        <v>498</v>
       </c>
     </row>
     <row r="149" spans="1:5">
       <c r="A149">
-        <v>148</v>
+        <v>147</v>
       </c>
       <c r="B149" t="s">
         <v>495</v>
@@ -5657,12 +5666,12 @@
         <v>497</v>
       </c>
       <c r="E149">
-        <v>496</v>
+        <v>492</v>
       </c>
     </row>
     <row r="150" spans="1:5">
       <c r="A150">
-        <v>149</v>
+        <v>148</v>
       </c>
       <c r="B150" t="s">
         <v>498</v>
@@ -5674,12 +5683,12 @@
         <v>500</v>
       </c>
       <c r="E150">
-        <v>499</v>
+        <v>496</v>
       </c>
     </row>
     <row r="151" spans="1:5">
       <c r="A151">
-        <v>150</v>
+        <v>149</v>
       </c>
       <c r="B151" t="s">
         <v>501</v>
@@ -5691,12 +5700,12 @@
         <v>503</v>
       </c>
       <c r="E151">
-        <v>500</v>
+        <v>499</v>
       </c>
     </row>
     <row r="152" spans="1:5">
       <c r="A152">
-        <v>151</v>
+        <v>150</v>
       </c>
       <c r="B152" t="s">
         <v>504</v>
@@ -5708,12 +5717,12 @@
         <v>506</v>
       </c>
       <c r="E152">
-        <v>504</v>
+        <v>500</v>
       </c>
     </row>
     <row r="153" spans="1:5">
       <c r="A153">
-        <v>152</v>
+        <v>151</v>
       </c>
       <c r="B153" t="s">
         <v>507</v>
@@ -5725,12 +5734,12 @@
         <v>509</v>
       </c>
       <c r="E153">
-        <v>508</v>
+        <v>504</v>
       </c>
     </row>
     <row r="154" spans="1:5">
       <c r="A154">
-        <v>153</v>
+        <v>152</v>
       </c>
       <c r="B154" t="s">
         <v>510</v>
@@ -5742,12 +5751,12 @@
         <v>512</v>
       </c>
       <c r="E154">
-        <v>104</v>
+        <v>508</v>
       </c>
     </row>
     <row r="155" spans="1:5">
       <c r="A155">
-        <v>154</v>
+        <v>153</v>
       </c>
       <c r="B155" t="s">
         <v>513</v>
@@ -5759,12 +5768,12 @@
         <v>515</v>
       </c>
       <c r="E155">
-        <v>516</v>
+        <v>104</v>
       </c>
     </row>
     <row r="156" spans="1:5">
       <c r="A156">
-        <v>155</v>
+        <v>154</v>
       </c>
       <c r="B156" t="s">
         <v>516</v>
@@ -5776,12 +5785,12 @@
         <v>518</v>
       </c>
       <c r="E156">
-        <v>520</v>
+        <v>516</v>
       </c>
     </row>
     <row r="157" spans="1:5">
       <c r="A157">
-        <v>156</v>
+        <v>155</v>
       </c>
       <c r="B157" t="s">
         <v>519</v>
@@ -5793,12 +5802,12 @@
         <v>521</v>
       </c>
       <c r="E157">
-        <v>524</v>
+        <v>520</v>
       </c>
     </row>
     <row r="158" spans="1:5">
       <c r="A158">
-        <v>157</v>
+        <v>156</v>
       </c>
       <c r="B158" t="s">
         <v>522</v>
@@ -5810,12 +5819,12 @@
         <v>524</v>
       </c>
       <c r="E158">
-        <v>528</v>
+        <v>524</v>
       </c>
     </row>
     <row r="159" spans="1:5">
       <c r="A159">
-        <v>158</v>
+        <v>157</v>
       </c>
       <c r="B159" t="s">
         <v>525</v>
@@ -5827,12 +5836,12 @@
         <v>527</v>
       </c>
       <c r="E159">
-        <v>540</v>
+        <v>528</v>
       </c>
     </row>
     <row r="160" spans="1:5">
       <c r="A160">
-        <v>159</v>
+        <v>158</v>
       </c>
       <c r="B160" t="s">
         <v>528</v>
@@ -5844,12 +5853,12 @@
         <v>530</v>
       </c>
       <c r="E160">
-        <v>554</v>
+        <v>540</v>
       </c>
     </row>
     <row r="161" spans="1:5">
       <c r="A161">
-        <v>160</v>
+        <v>159</v>
       </c>
       <c r="B161" t="s">
         <v>531</v>
@@ -5861,12 +5870,12 @@
         <v>533</v>
       </c>
       <c r="E161">
-        <v>558</v>
+        <v>554</v>
       </c>
     </row>
     <row r="162" spans="1:5">
       <c r="A162">
-        <v>161</v>
+        <v>160</v>
       </c>
       <c r="B162" t="s">
         <v>534</v>
@@ -5878,12 +5887,12 @@
         <v>536</v>
       </c>
       <c r="E162">
-        <v>562</v>
+        <v>558</v>
       </c>
     </row>
     <row r="163" spans="1:5">
       <c r="A163">
-        <v>162</v>
+        <v>161</v>
       </c>
       <c r="B163" t="s">
         <v>537</v>
@@ -5895,12 +5904,12 @@
         <v>539</v>
       </c>
       <c r="E163">
-        <v>566</v>
+        <v>562</v>
       </c>
     </row>
     <row r="164" spans="1:5">
       <c r="A164">
-        <v>163</v>
+        <v>162</v>
       </c>
       <c r="B164" t="s">
         <v>540</v>
@@ -5912,12 +5921,12 @@
         <v>542</v>
       </c>
       <c r="E164">
-        <v>570</v>
+        <v>566</v>
       </c>
     </row>
     <row r="165" spans="1:5">
       <c r="A165">
-        <v>164</v>
+        <v>163</v>
       </c>
       <c r="B165" t="s">
         <v>543</v>
@@ -5929,12 +5938,12 @@
         <v>545</v>
       </c>
       <c r="E165">
-        <v>574</v>
+        <v>570</v>
       </c>
     </row>
     <row r="166" spans="1:5">
       <c r="A166">
-        <v>132</v>
+        <v>164</v>
       </c>
       <c r="B166" t="s">
         <v>546</v>
@@ -5946,12 +5955,12 @@
         <v>548</v>
       </c>
       <c r="E166">
-        <v>807</v>
+        <v>574</v>
       </c>
     </row>
     <row r="167" spans="1:5">
       <c r="A167">
-        <v>165</v>
+        <v>132</v>
       </c>
       <c r="B167" t="s">
         <v>549</v>
@@ -5963,12 +5972,12 @@
         <v>551</v>
       </c>
       <c r="E167">
-        <v>580</v>
+        <v>807</v>
       </c>
     </row>
     <row r="168" spans="1:5">
       <c r="A168">
-        <v>166</v>
+        <v>165</v>
       </c>
       <c r="B168" t="s">
         <v>552</v>
@@ -5980,12 +5989,12 @@
         <v>554</v>
       </c>
       <c r="E168">
-        <v>578</v>
+        <v>580</v>
       </c>
     </row>
     <row r="169" spans="1:5">
       <c r="A169">
-        <v>167</v>
+        <v>166</v>
       </c>
       <c r="B169" t="s">
         <v>555</v>
@@ -5997,12 +6006,12 @@
         <v>557</v>
       </c>
       <c r="E169">
-        <v>512</v>
+        <v>578</v>
       </c>
     </row>
     <row r="170" spans="1:5">
       <c r="A170">
-        <v>168</v>
+        <v>167</v>
       </c>
       <c r="B170" t="s">
         <v>558</v>
@@ -6014,12 +6023,12 @@
         <v>560</v>
       </c>
       <c r="E170">
-        <v>586</v>
+        <v>512</v>
       </c>
     </row>
     <row r="171" spans="1:5">
       <c r="A171">
-        <v>169</v>
+        <v>168</v>
       </c>
       <c r="B171" t="s">
         <v>561</v>
@@ -6031,12 +6040,12 @@
         <v>563</v>
       </c>
       <c r="E171">
-        <v>585</v>
+        <v>586</v>
       </c>
     </row>
     <row r="172" spans="1:5">
       <c r="A172">
-        <v>170</v>
+        <v>169</v>
       </c>
       <c r="B172" t="s">
         <v>564</v>
@@ -6048,12 +6057,12 @@
         <v>566</v>
       </c>
       <c r="E172">
-        <v>275</v>
+        <v>585</v>
       </c>
     </row>
     <row r="173" spans="1:5">
       <c r="A173">
-        <v>171</v>
+        <v>170</v>
       </c>
       <c r="B173" t="s">
         <v>567</v>
@@ -6065,12 +6074,12 @@
         <v>569</v>
       </c>
       <c r="E173">
-        <v>591</v>
+        <v>275</v>
       </c>
     </row>
     <row r="174" spans="1:5">
       <c r="A174">
-        <v>172</v>
+        <v>171</v>
       </c>
       <c r="B174" t="s">
         <v>570</v>
@@ -6082,12 +6091,12 @@
         <v>572</v>
       </c>
       <c r="E174">
-        <v>598</v>
+        <v>591</v>
       </c>
     </row>
     <row r="175" spans="1:5">
       <c r="A175">
-        <v>173</v>
+        <v>172</v>
       </c>
       <c r="B175" t="s">
         <v>573</v>
@@ -6099,12 +6108,12 @@
         <v>575</v>
       </c>
       <c r="E175">
-        <v>600</v>
+        <v>598</v>
       </c>
     </row>
     <row r="176" spans="1:5">
       <c r="A176">
-        <v>174</v>
+        <v>173</v>
       </c>
       <c r="B176" t="s">
         <v>576</v>
@@ -6116,12 +6125,12 @@
         <v>578</v>
       </c>
       <c r="E176">
-        <v>604</v>
+        <v>600</v>
       </c>
     </row>
     <row r="177" spans="1:5">
       <c r="A177">
-        <v>175</v>
+        <v>174</v>
       </c>
       <c r="B177" t="s">
         <v>579</v>
@@ -6133,12 +6142,12 @@
         <v>581</v>
       </c>
       <c r="E177">
-        <v>608</v>
+        <v>604</v>
       </c>
     </row>
     <row r="178" spans="1:5">
       <c r="A178">
-        <v>176</v>
+        <v>175</v>
       </c>
       <c r="B178" t="s">
         <v>582</v>
@@ -6150,12 +6159,12 @@
         <v>584</v>
       </c>
       <c r="E178">
-        <v>612</v>
+        <v>608</v>
       </c>
     </row>
     <row r="179" spans="1:5">
       <c r="A179">
-        <v>177</v>
+        <v>176</v>
       </c>
       <c r="B179" t="s">
         <v>585</v>
@@ -6167,12 +6176,12 @@
         <v>587</v>
       </c>
       <c r="E179">
-        <v>616</v>
+        <v>612</v>
       </c>
     </row>
     <row r="180" spans="1:5">
       <c r="A180">
-        <v>178</v>
+        <v>177</v>
       </c>
       <c r="B180" t="s">
         <v>588</v>
@@ -6184,12 +6193,12 @@
         <v>590</v>
       </c>
       <c r="E180">
-        <v>620</v>
+        <v>616</v>
       </c>
     </row>
     <row r="181" spans="1:5">
       <c r="A181">
-        <v>179</v>
+        <v>178</v>
       </c>
       <c r="B181" t="s">
         <v>591</v>
@@ -6201,12 +6210,12 @@
         <v>593</v>
       </c>
       <c r="E181">
-        <v>630</v>
+        <v>620</v>
       </c>
     </row>
     <row r="182" spans="1:5">
       <c r="A182">
-        <v>180</v>
+        <v>179</v>
       </c>
       <c r="B182" t="s">
         <v>594</v>
@@ -6218,12 +6227,12 @@
         <v>596</v>
       </c>
       <c r="E182">
-        <v>634</v>
+        <v>630</v>
       </c>
     </row>
     <row r="183" spans="1:5">
       <c r="A183">
-        <v>181</v>
+        <v>180</v>
       </c>
       <c r="B183" t="s">
         <v>597</v>
@@ -6235,12 +6244,12 @@
         <v>599</v>
       </c>
       <c r="E183">
-        <v>638</v>
+        <v>634</v>
       </c>
     </row>
     <row r="184" spans="1:5">
       <c r="A184">
-        <v>182</v>
+        <v>181</v>
       </c>
       <c r="B184" t="s">
         <v>600</v>
@@ -6252,12 +6261,12 @@
         <v>602</v>
       </c>
       <c r="E184">
-        <v>642</v>
+        <v>638</v>
       </c>
     </row>
     <row r="185" spans="1:5">
       <c r="A185">
-        <v>183</v>
+        <v>182</v>
       </c>
       <c r="B185" t="s">
         <v>603</v>
@@ -6269,12 +6278,12 @@
         <v>605</v>
       </c>
       <c r="E185">
-        <v>643</v>
+        <v>642</v>
       </c>
     </row>
     <row r="186" spans="1:5">
       <c r="A186">
-        <v>184</v>
+        <v>183</v>
       </c>
       <c r="B186" t="s">
         <v>606</v>
@@ -6286,12 +6295,12 @@
         <v>608</v>
       </c>
       <c r="E186">
-        <v>646</v>
+        <v>643</v>
       </c>
     </row>
     <row r="187" spans="1:5">
       <c r="A187">
-        <v>185</v>
+        <v>184</v>
       </c>
       <c r="B187" t="s">
         <v>609</v>
@@ -6303,12 +6312,12 @@
         <v>611</v>
       </c>
       <c r="E187">
-        <v>652</v>
+        <v>646</v>
       </c>
     </row>
     <row r="188" spans="1:5">
       <c r="A188">
-        <v>186</v>
+        <v>185</v>
       </c>
       <c r="B188" t="s">
         <v>612</v>
@@ -6320,12 +6329,12 @@
         <v>614</v>
       </c>
       <c r="E188">
-        <v>654</v>
+        <v>652</v>
       </c>
     </row>
     <row r="189" spans="1:5">
       <c r="A189">
-        <v>187</v>
+        <v>186</v>
       </c>
       <c r="B189" t="s">
         <v>615</v>
@@ -6337,12 +6346,12 @@
         <v>617</v>
       </c>
       <c r="E189">
-        <v>659</v>
+        <v>654</v>
       </c>
     </row>
     <row r="190" spans="1:5">
       <c r="A190">
-        <v>188</v>
+        <v>187</v>
       </c>
       <c r="B190" t="s">
         <v>618</v>
@@ -6354,12 +6363,12 @@
         <v>620</v>
       </c>
       <c r="E190">
-        <v>662</v>
+        <v>659</v>
       </c>
     </row>
     <row r="191" spans="1:5">
       <c r="A191">
-        <v>189</v>
+        <v>188</v>
       </c>
       <c r="B191" t="s">
         <v>621</v>
@@ -6371,12 +6380,12 @@
         <v>623</v>
       </c>
       <c r="E191">
-        <v>663</v>
+        <v>662</v>
       </c>
     </row>
     <row r="192" spans="1:5">
       <c r="A192">
-        <v>190</v>
+        <v>189</v>
       </c>
       <c r="B192" t="s">
         <v>624</v>
@@ -6388,12 +6397,12 @@
         <v>626</v>
       </c>
       <c r="E192">
-        <v>666</v>
+        <v>663</v>
       </c>
     </row>
     <row r="193" spans="1:5">
       <c r="A193">
-        <v>191</v>
+        <v>190</v>
       </c>
       <c r="B193" t="s">
         <v>627</v>
@@ -6405,12 +6414,12 @@
         <v>629</v>
       </c>
       <c r="E193">
-        <v>670</v>
+        <v>666</v>
       </c>
     </row>
     <row r="194" spans="1:5">
       <c r="A194">
-        <v>192</v>
+        <v>191</v>
       </c>
       <c r="B194" t="s">
         <v>630</v>
@@ -6422,12 +6431,12 @@
         <v>632</v>
       </c>
       <c r="E194">
-        <v>882</v>
+        <v>670</v>
       </c>
     </row>
     <row r="195" spans="1:5">
       <c r="A195">
-        <v>193</v>
+        <v>192</v>
       </c>
       <c r="B195" t="s">
         <v>633</v>
@@ -6439,12 +6448,12 @@
         <v>635</v>
       </c>
       <c r="E195">
-        <v>674</v>
+        <v>882</v>
       </c>
     </row>
     <row r="196" spans="1:5">
       <c r="A196">
-        <v>194</v>
+        <v>193</v>
       </c>
       <c r="B196" t="s">
         <v>636</v>
@@ -6456,12 +6465,12 @@
         <v>638</v>
       </c>
       <c r="E196">
-        <v>678</v>
+        <v>674</v>
       </c>
     </row>
     <row r="197" spans="1:5">
       <c r="A197">
-        <v>195</v>
+        <v>194</v>
       </c>
       <c r="B197" t="s">
         <v>639</v>
@@ -6473,12 +6482,12 @@
         <v>641</v>
       </c>
       <c r="E197">
-        <v>682</v>
+        <v>678</v>
       </c>
     </row>
     <row r="198" spans="1:5">
       <c r="A198">
-        <v>196</v>
+        <v>195</v>
       </c>
       <c r="B198" t="s">
         <v>642</v>
@@ -6490,12 +6499,12 @@
         <v>644</v>
       </c>
       <c r="E198">
-        <v>686</v>
+        <v>682</v>
       </c>
     </row>
     <row r="199" spans="1:5">
       <c r="A199">
-        <v>197</v>
+        <v>196</v>
       </c>
       <c r="B199" t="s">
         <v>645</v>
@@ -6507,12 +6516,12 @@
         <v>647</v>
       </c>
       <c r="E199">
-        <v>688</v>
+        <v>686</v>
       </c>
     </row>
     <row r="200" spans="1:5">
       <c r="A200">
-        <v>198</v>
+        <v>197</v>
       </c>
       <c r="B200" t="s">
         <v>648</v>
@@ -6524,12 +6533,12 @@
         <v>650</v>
       </c>
       <c r="E200">
-        <v>690</v>
+        <v>688</v>
       </c>
     </row>
     <row r="201" spans="1:5">
       <c r="A201">
-        <v>199</v>
+        <v>198</v>
       </c>
       <c r="B201" t="s">
         <v>651</v>
@@ -6541,12 +6550,12 @@
         <v>653</v>
       </c>
       <c r="E201">
-        <v>694</v>
+        <v>690</v>
       </c>
     </row>
     <row r="202" spans="1:5">
       <c r="A202">
-        <v>200</v>
+        <v>199</v>
       </c>
       <c r="B202" t="s">
         <v>654</v>
@@ -6558,12 +6567,12 @@
         <v>656</v>
       </c>
       <c r="E202">
-        <v>702</v>
+        <v>694</v>
       </c>
     </row>
     <row r="203" spans="1:5">
       <c r="A203">
-        <v>201</v>
+        <v>200</v>
       </c>
       <c r="B203" t="s">
         <v>657</v>
@@ -6575,12 +6584,12 @@
         <v>659</v>
       </c>
       <c r="E203">
-        <v>534</v>
+        <v>702</v>
       </c>
     </row>
     <row r="204" spans="1:5">
       <c r="A204">
-        <v>202</v>
+        <v>201</v>
       </c>
       <c r="B204" t="s">
         <v>660</v>
@@ -6592,12 +6601,12 @@
         <v>662</v>
       </c>
       <c r="E204">
-        <v>703</v>
+        <v>534</v>
       </c>
     </row>
     <row r="205" spans="1:5">
       <c r="A205">
-        <v>203</v>
+        <v>202</v>
       </c>
       <c r="B205" t="s">
         <v>663</v>
@@ -6609,12 +6618,12 @@
         <v>665</v>
       </c>
       <c r="E205">
-        <v>705</v>
+        <v>703</v>
       </c>
     </row>
     <row r="206" spans="1:5">
       <c r="A206">
-        <v>204</v>
+        <v>203</v>
       </c>
       <c r="B206" t="s">
         <v>666</v>
@@ -6626,12 +6635,12 @@
         <v>668</v>
       </c>
       <c r="E206">
-        <v>90</v>
+        <v>705</v>
       </c>
     </row>
     <row r="207" spans="1:5">
       <c r="A207">
-        <v>205</v>
+        <v>204</v>
       </c>
       <c r="B207" t="s">
         <v>669</v>
@@ -6643,12 +6652,12 @@
         <v>671</v>
       </c>
       <c r="E207">
-        <v>706</v>
+        <v>90</v>
       </c>
     </row>
     <row r="208" spans="1:5">
       <c r="A208">
-        <v>206</v>
+        <v>205</v>
       </c>
       <c r="B208" t="s">
         <v>672</v>
@@ -6660,12 +6669,12 @@
         <v>674</v>
       </c>
       <c r="E208">
-        <v>710</v>
+        <v>706</v>
       </c>
     </row>
     <row r="209" spans="1:5">
       <c r="A209">
-        <v>207</v>
+        <v>206</v>
       </c>
       <c r="B209" t="s">
         <v>675</v>
@@ -6677,12 +6686,12 @@
         <v>677</v>
       </c>
       <c r="E209">
-        <v>239</v>
+        <v>710</v>
       </c>
     </row>
     <row r="210" spans="1:5">
       <c r="A210">
-        <v>208</v>
+        <v>207</v>
       </c>
       <c r="B210" t="s">
         <v>678</v>
@@ -6694,12 +6703,12 @@
         <v>680</v>
       </c>
       <c r="E210">
-        <v>728</v>
+        <v>239</v>
       </c>
     </row>
     <row r="211" spans="1:5">
       <c r="A211">
-        <v>209</v>
+        <v>208</v>
       </c>
       <c r="B211" t="s">
         <v>681</v>
@@ -6711,12 +6720,12 @@
         <v>683</v>
       </c>
       <c r="E211">
-        <v>724</v>
+        <v>728</v>
       </c>
     </row>
     <row r="212" spans="1:5">
       <c r="A212">
-        <v>210</v>
+        <v>209</v>
       </c>
       <c r="B212" t="s">
         <v>684</v>
@@ -6728,12 +6737,12 @@
         <v>686</v>
       </c>
       <c r="E212">
-        <v>144</v>
+        <v>724</v>
       </c>
     </row>
     <row r="213" spans="1:5">
       <c r="A213">
-        <v>211</v>
+        <v>210</v>
       </c>
       <c r="B213" t="s">
         <v>687</v>
@@ -6745,12 +6754,12 @@
         <v>689</v>
       </c>
       <c r="E213">
-        <v>729</v>
+        <v>144</v>
       </c>
     </row>
     <row r="214" spans="1:5">
       <c r="A214">
-        <v>212</v>
+        <v>211</v>
       </c>
       <c r="B214" t="s">
         <v>690</v>
@@ -6762,12 +6771,12 @@
         <v>692</v>
       </c>
       <c r="E214">
-        <v>740</v>
+        <v>729</v>
       </c>
     </row>
     <row r="215" spans="1:5">
       <c r="A215">
-        <v>213</v>
+        <v>212</v>
       </c>
       <c r="B215" t="s">
         <v>693</v>
@@ -6779,12 +6788,12 @@
         <v>695</v>
       </c>
       <c r="E215">
-        <v>744</v>
+        <v>740</v>
       </c>
     </row>
     <row r="216" spans="1:5">
       <c r="A216">
-        <v>215</v>
+        <v>213</v>
       </c>
       <c r="B216" t="s">
         <v>696</v>
@@ -6796,12 +6805,12 @@
         <v>698</v>
       </c>
       <c r="E216">
-        <v>752</v>
+        <v>744</v>
       </c>
     </row>
     <row r="217" spans="1:5">
       <c r="A217">
-        <v>216</v>
+        <v>215</v>
       </c>
       <c r="B217" t="s">
         <v>699</v>
@@ -6813,12 +6822,12 @@
         <v>701</v>
       </c>
       <c r="E217">
-        <v>756</v>
+        <v>752</v>
       </c>
     </row>
     <row r="218" spans="1:5">
       <c r="A218">
-        <v>217</v>
+        <v>216</v>
       </c>
       <c r="B218" t="s">
         <v>702</v>
@@ -6830,12 +6839,12 @@
         <v>704</v>
       </c>
       <c r="E218">
-        <v>760</v>
+        <v>756</v>
       </c>
     </row>
     <row r="219" spans="1:5">
       <c r="A219">
-        <v>218</v>
+        <v>217</v>
       </c>
       <c r="B219" t="s">
         <v>705</v>
@@ -6847,12 +6856,12 @@
         <v>707</v>
       </c>
       <c r="E219">
-        <v>158</v>
+        <v>760</v>
       </c>
     </row>
     <row r="220" spans="1:5">
       <c r="A220">
-        <v>219</v>
+        <v>218</v>
       </c>
       <c r="B220" t="s">
         <v>708</v>
@@ -6864,12 +6873,12 @@
         <v>710</v>
       </c>
       <c r="E220">
-        <v>762</v>
+        <v>158</v>
       </c>
     </row>
     <row r="221" spans="1:5">
       <c r="A221">
-        <v>220</v>
+        <v>219</v>
       </c>
       <c r="B221" t="s">
         <v>711</v>
@@ -6881,12 +6890,12 @@
         <v>713</v>
       </c>
       <c r="E221">
-        <v>834</v>
+        <v>762</v>
       </c>
     </row>
     <row r="222" spans="1:5">
       <c r="A222">
-        <v>221</v>
+        <v>220</v>
       </c>
       <c r="B222" t="s">
         <v>714</v>
@@ -6898,12 +6907,12 @@
         <v>716</v>
       </c>
       <c r="E222">
-        <v>764</v>
+        <v>834</v>
       </c>
     </row>
     <row r="223" spans="1:5">
       <c r="A223">
-        <v>222</v>
+        <v>221</v>
       </c>
       <c r="B223" t="s">
         <v>717</v>
@@ -6915,12 +6924,12 @@
         <v>719</v>
       </c>
       <c r="E223">
-        <v>626</v>
+        <v>764</v>
       </c>
     </row>
     <row r="224" spans="1:5">
       <c r="A224">
-        <v>223</v>
+        <v>222</v>
       </c>
       <c r="B224" t="s">
         <v>720</v>
@@ -6932,12 +6941,12 @@
         <v>722</v>
       </c>
       <c r="E224">
-        <v>768</v>
+        <v>626</v>
       </c>
     </row>
     <row r="225" spans="1:5">
       <c r="A225">
-        <v>224</v>
+        <v>223</v>
       </c>
       <c r="B225" t="s">
         <v>723</v>
@@ -6949,12 +6958,12 @@
         <v>725</v>
       </c>
       <c r="E225">
-        <v>772</v>
+        <v>768</v>
       </c>
     </row>
     <row r="226" spans="1:5">
       <c r="A226">
-        <v>225</v>
+        <v>224</v>
       </c>
       <c r="B226" t="s">
         <v>726</v>
@@ -6966,12 +6975,12 @@
         <v>728</v>
       </c>
       <c r="E226">
-        <v>776</v>
+        <v>772</v>
       </c>
     </row>
     <row r="227" spans="1:5">
       <c r="A227">
-        <v>226</v>
+        <v>225</v>
       </c>
       <c r="B227" t="s">
         <v>729</v>
@@ -6983,46 +6992,46 @@
         <v>731</v>
       </c>
       <c r="E227">
-        <v>780</v>
+        <v>776</v>
       </c>
     </row>
     <row r="228" spans="1:5">
       <c r="A228">
-        <v>227</v>
+        <v>226</v>
       </c>
       <c r="B228" t="s">
         <v>732</v>
       </c>
       <c r="C228" t="s">
-        <v>48</v>
+        <v>733</v>
       </c>
       <c r="D228" t="s">
-        <v>733</v>
+        <v>734</v>
       </c>
       <c r="E228">
-        <v>788</v>
+        <v>780</v>
       </c>
     </row>
     <row r="229" spans="1:5">
       <c r="A229">
-        <v>228</v>
+        <v>227</v>
       </c>
       <c r="B229" t="s">
-        <v>734</v>
+        <v>735</v>
       </c>
       <c r="C229" t="s">
-        <v>735</v>
+        <v>48</v>
       </c>
       <c r="D229" t="s">
         <v>736</v>
       </c>
       <c r="E229">
-        <v>792</v>
+        <v>788</v>
       </c>
     </row>
     <row r="230" spans="1:5">
       <c r="A230">
-        <v>229</v>
+        <v>228</v>
       </c>
       <c r="B230" t="s">
         <v>737</v>
@@ -7034,12 +7043,12 @@
         <v>739</v>
       </c>
       <c r="E230">
-        <v>795</v>
+        <v>792</v>
       </c>
     </row>
     <row r="231" spans="1:5">
       <c r="A231">
-        <v>230</v>
+        <v>229</v>
       </c>
       <c r="B231" t="s">
         <v>740</v>
@@ -7051,12 +7060,12 @@
         <v>742</v>
       </c>
       <c r="E231">
-        <v>796</v>
+        <v>795</v>
       </c>
     </row>
     <row r="232" spans="1:5">
       <c r="A232">
-        <v>231</v>
+        <v>230</v>
       </c>
       <c r="B232" t="s">
         <v>743</v>
@@ -7068,12 +7077,12 @@
         <v>745</v>
       </c>
       <c r="E232">
-        <v>798</v>
+        <v>796</v>
       </c>
     </row>
     <row r="233" spans="1:5">
       <c r="A233">
-        <v>232</v>
+        <v>231</v>
       </c>
       <c r="B233" t="s">
         <v>746</v>
@@ -7085,12 +7094,12 @@
         <v>748</v>
       </c>
       <c r="E233">
-        <v>800</v>
+        <v>798</v>
       </c>
     </row>
     <row r="234" spans="1:5">
       <c r="A234">
-        <v>233</v>
+        <v>232</v>
       </c>
       <c r="B234" t="s">
         <v>749</v>
@@ -7102,12 +7111,12 @@
         <v>751</v>
       </c>
       <c r="E234">
-        <v>804</v>
+        <v>800</v>
       </c>
     </row>
     <row r="235" spans="1:5">
       <c r="A235">
-        <v>234</v>
+        <v>233</v>
       </c>
       <c r="B235" t="s">
         <v>752</v>
@@ -7119,12 +7128,12 @@
         <v>754</v>
       </c>
       <c r="E235">
-        <v>784</v>
+        <v>804</v>
       </c>
     </row>
     <row r="236" spans="1:5">
       <c r="A236">
-        <v>235</v>
+        <v>234</v>
       </c>
       <c r="B236" t="s">
         <v>755</v>
@@ -7136,12 +7145,12 @@
         <v>757</v>
       </c>
       <c r="E236">
-        <v>826</v>
+        <v>784</v>
       </c>
     </row>
     <row r="237" spans="1:5">
       <c r="A237">
-        <v>236</v>
+        <v>235</v>
       </c>
       <c r="B237" t="s">
         <v>758</v>
@@ -7153,12 +7162,12 @@
         <v>760</v>
       </c>
       <c r="E237">
-        <v>840</v>
+        <v>826</v>
       </c>
     </row>
     <row r="238" spans="1:5">
       <c r="A238">
-        <v>237</v>
+        <v>236</v>
       </c>
       <c r="B238" t="s">
         <v>761</v>
@@ -7170,12 +7179,12 @@
         <v>763</v>
       </c>
       <c r="E238">
-        <v>581</v>
+        <v>840</v>
       </c>
     </row>
     <row r="239" spans="1:5">
       <c r="A239">
-        <v>238</v>
+        <v>237</v>
       </c>
       <c r="B239" t="s">
         <v>764</v>
@@ -7187,12 +7196,12 @@
         <v>766</v>
       </c>
       <c r="E239">
-        <v>858</v>
+        <v>581</v>
       </c>
     </row>
     <row r="240" spans="1:5">
       <c r="A240">
-        <v>239</v>
+        <v>238</v>
       </c>
       <c r="B240" t="s">
         <v>767</v>
@@ -7204,12 +7213,12 @@
         <v>769</v>
       </c>
       <c r="E240">
-        <v>860</v>
+        <v>858</v>
       </c>
     </row>
     <row r="241" spans="1:5">
       <c r="A241">
-        <v>240</v>
+        <v>239</v>
       </c>
       <c r="B241" t="s">
         <v>770</v>
@@ -7221,12 +7230,12 @@
         <v>772</v>
       </c>
       <c r="E241">
-        <v>548</v>
+        <v>860</v>
       </c>
     </row>
     <row r="242" spans="1:5">
       <c r="A242">
-        <v>241</v>
+        <v>240</v>
       </c>
       <c r="B242" t="s">
         <v>773</v>
@@ -7238,12 +7247,12 @@
         <v>775</v>
       </c>
       <c r="E242">
-        <v>862</v>
+        <v>548</v>
       </c>
     </row>
     <row r="243" spans="1:5">
       <c r="A243">
-        <v>242</v>
+        <v>241</v>
       </c>
       <c r="B243" t="s">
         <v>776</v>
@@ -7255,12 +7264,12 @@
         <v>778</v>
       </c>
       <c r="E243">
-        <v>704</v>
+        <v>862</v>
       </c>
     </row>
     <row r="244" spans="1:5">
       <c r="A244">
-        <v>243</v>
+        <v>242</v>
       </c>
       <c r="B244" t="s">
         <v>779</v>
@@ -7272,12 +7281,12 @@
         <v>781</v>
       </c>
       <c r="E244">
-        <v>92</v>
+        <v>704</v>
       </c>
     </row>
     <row r="245" spans="1:5">
       <c r="A245">
-        <v>244</v>
+        <v>243</v>
       </c>
       <c r="B245" t="s">
         <v>782</v>
@@ -7289,12 +7298,12 @@
         <v>784</v>
       </c>
       <c r="E245">
-        <v>850</v>
+        <v>92</v>
       </c>
     </row>
     <row r="246" spans="1:5">
       <c r="A246">
-        <v>245</v>
+        <v>244</v>
       </c>
       <c r="B246" t="s">
         <v>785</v>
@@ -7306,12 +7315,12 @@
         <v>787</v>
       </c>
       <c r="E246">
-        <v>876</v>
+        <v>850</v>
       </c>
     </row>
     <row r="247" spans="1:5">
       <c r="A247">
-        <v>246</v>
+        <v>245</v>
       </c>
       <c r="B247" t="s">
         <v>788</v>
@@ -7323,12 +7332,12 @@
         <v>790</v>
       </c>
       <c r="E247">
-        <v>732</v>
+        <v>876</v>
       </c>
     </row>
     <row r="248" spans="1:5">
       <c r="A248">
-        <v>247</v>
+        <v>246</v>
       </c>
       <c r="B248" t="s">
         <v>791</v>
@@ -7340,12 +7349,12 @@
         <v>793</v>
       </c>
       <c r="E248">
-        <v>887</v>
+        <v>732</v>
       </c>
     </row>
     <row r="249" spans="1:5">
       <c r="A249">
-        <v>248</v>
+        <v>247</v>
       </c>
       <c r="B249" t="s">
         <v>794</v>
@@ -7357,12 +7366,12 @@
         <v>796</v>
       </c>
       <c r="E249">
-        <v>894</v>
+        <v>887</v>
       </c>
     </row>
     <row r="250" spans="1:5">
       <c r="A250">
-        <v>249</v>
+        <v>248</v>
       </c>
       <c r="B250" t="s">
         <v>797</v>
@@ -7374,6 +7383,23 @@
         <v>799</v>
       </c>
       <c r="E250">
+        <v>894</v>
+      </c>
+    </row>
+    <row r="251" spans="1:5">
+      <c r="A251">
+        <v>249</v>
+      </c>
+      <c r="B251" t="s">
+        <v>800</v>
+      </c>
+      <c r="C251" t="s">
+        <v>801</v>
+      </c>
+      <c r="D251" t="s">
+        <v>802</v>
+      </c>
+      <c r="E251">
         <v>716</v>
       </c>
     </row>

</xml_diff>